<commit_message>
Fix RFI reports description missing, error log strikeout, and add full details to error email updates
</commit_message>
<xml_diff>
--- a/backend/test.xlsx
+++ b/backend/test.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="SOW" state="visible" r:id="rId3"/>
+    <sheet sheetId="1" name="RFI LOG" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -12,19 +12,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-    </font>
-    <font>
-      <u/>
     </font>
   </fonts>
   <fills count="2">
@@ -47,10 +41,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -66,6 +58,50 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3333750" cy="714375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -390,17 +426,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>